<commit_message>
feat: updates UI config badges, data parsing aggregation for 1967 scenario, and fixes translations
This commit addresses KeyError issues on CSV BOM parsing, adds fallback string splitting for historical role aggregations, and standardizes scientific terminology for legacy roles. Modifies UI to render configuration badges on views 1 and 2.
</commit_message>
<xml_diff>
--- a/11 - Atrib Decreto 47788-1967 original.xlsx
+++ b/11 - Atrib Decreto 47788-1967 original.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiap\OneDrive\Desktop\Desenvolvimento\Estudo_Atribuicoes_PCSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C07CF26-9F23-4C60-A771-E4A13CACECCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD20993-39F8-4ED7-A908-948DB94A1A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{9E2F6A9B-94A3-41DD-92E9-2C4405031CDE}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Delegado de Polícia</t>
   </si>
@@ -122,6 +122,30 @@
   </si>
   <si>
     <t>manipulação de ossos e partes do corpo</t>
+  </si>
+  <si>
+    <t>Escrivão de Polícia</t>
+  </si>
+  <si>
+    <t>Organização de Inquérito</t>
+  </si>
+  <si>
+    <t>atuar na investigação</t>
+  </si>
+  <si>
+    <t>Licenciamento e Registro</t>
+  </si>
+  <si>
+    <t>Manutenção de Escritório</t>
+  </si>
+  <si>
+    <t>Investigador de Policia</t>
+  </si>
+  <si>
+    <t>policiamento e prevenção de crime</t>
+  </si>
+  <si>
+    <t>cumprir mandados</t>
   </si>
 </sst>
 </file>
@@ -1027,90 +1051,110 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E66DEB-712A-465C-882E-F5424BC162B6}">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="30.109375" customWidth="1"/>
-    <col min="14" max="14" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="22" width="30.77734375" customWidth="1"/>
+    <col min="2" max="2" width="32.21875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="29.77734375" customWidth="1"/>
+    <col min="9" max="9" width="29" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="19" width="30.109375" customWidth="1"/>
+    <col min="20" max="20" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="28" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1177,757 +1221,1145 @@
       <c r="V2" s="4">
         <v>0</v>
       </c>
+      <c r="W2" s="4">
+        <v>0</v>
+      </c>
+      <c r="X2" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>1</v>
+      </c>
+      <c r="J3" s="4">
+        <v>1</v>
+      </c>
+      <c r="K3" s="4">
+        <v>1</v>
+      </c>
+      <c r="L3" s="4">
+        <v>1</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4">
+        <v>0</v>
+      </c>
+      <c r="T3" s="4">
+        <v>0</v>
+      </c>
+      <c r="U3" s="4">
+        <v>0</v>
+      </c>
+      <c r="V3" s="4">
+        <v>0</v>
+      </c>
+      <c r="W3" s="4">
+        <v>0</v>
+      </c>
+      <c r="X3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="4">
+        <v>1</v>
+      </c>
+      <c r="L4" s="4">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4">
+        <v>0</v>
+      </c>
+      <c r="T4" s="4">
+        <v>0</v>
+      </c>
+      <c r="U4" s="4">
+        <v>0</v>
+      </c>
+      <c r="V4" s="4">
+        <v>0</v>
+      </c>
+      <c r="W4" s="4">
+        <v>0</v>
+      </c>
+      <c r="X4" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4">
-        <v>1</v>
-      </c>
-      <c r="D3" s="4">
-        <v>1</v>
-      </c>
-      <c r="E3" s="4">
-        <v>1</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4">
-        <v>0</v>
-      </c>
-      <c r="I3" s="4">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4">
-        <v>0</v>
-      </c>
-      <c r="K3" s="4">
-        <v>0</v>
-      </c>
-      <c r="L3" s="4">
-        <v>0</v>
-      </c>
-      <c r="M3" s="4">
-        <v>0</v>
-      </c>
-      <c r="N3" s="4">
-        <v>0</v>
-      </c>
-      <c r="O3" s="4">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="4">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4">
-        <v>0</v>
-      </c>
-      <c r="T3" s="4">
-        <v>0</v>
-      </c>
-      <c r="U3" s="4">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4">
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>1</v>
+      </c>
+      <c r="J5" s="4">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4">
+        <v>1</v>
+      </c>
+      <c r="L5" s="4">
+        <v>1</v>
+      </c>
+      <c r="M5" s="4">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>0</v>
+      </c>
+      <c r="R5" s="4">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4">
+        <v>0</v>
+      </c>
+      <c r="T5" s="4">
+        <v>0</v>
+      </c>
+      <c r="U5" s="4">
+        <v>0</v>
+      </c>
+      <c r="V5" s="4">
+        <v>0</v>
+      </c>
+      <c r="W5" s="4">
+        <v>0</v>
+      </c>
+      <c r="X5" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4">
-        <v>1</v>
-      </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4">
-        <v>0</v>
-      </c>
-      <c r="M4" s="4">
-        <v>0</v>
-      </c>
-      <c r="N4" s="4">
-        <v>0</v>
-      </c>
-      <c r="O4" s="4">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4">
-        <v>0</v>
-      </c>
-      <c r="V4" s="4">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4">
+        <v>1</v>
+      </c>
+      <c r="N6" s="4">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4">
+        <v>0</v>
+      </c>
+      <c r="T6" s="4">
+        <v>0</v>
+      </c>
+      <c r="U6" s="4">
+        <v>0</v>
+      </c>
+      <c r="V6" s="4">
+        <v>0</v>
+      </c>
+      <c r="W6" s="4">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4">
-        <v>1</v>
-      </c>
-      <c r="I5" s="4">
-        <v>1</v>
-      </c>
-      <c r="J5" s="4">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4">
-        <v>0</v>
-      </c>
-      <c r="M5" s="4">
-        <v>0</v>
-      </c>
-      <c r="N5" s="4">
-        <v>0</v>
-      </c>
-      <c r="O5" s="4">
-        <v>0</v>
-      </c>
-      <c r="P5" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="4">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4">
-        <v>0</v>
-      </c>
-      <c r="T5" s="4">
-        <v>0</v>
-      </c>
-      <c r="U5" s="4">
-        <v>0</v>
-      </c>
-      <c r="V5" s="4">
+      <c r="B7" s="4">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4">
+        <v>1</v>
+      </c>
+      <c r="O7" s="4">
+        <v>1</v>
+      </c>
+      <c r="P7" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4">
+        <v>0</v>
+      </c>
+      <c r="R7" s="4">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4">
+        <v>0</v>
+      </c>
+      <c r="T7" s="4">
+        <v>0</v>
+      </c>
+      <c r="U7" s="4">
+        <v>0</v>
+      </c>
+      <c r="V7" s="4">
+        <v>0</v>
+      </c>
+      <c r="W7" s="4">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4">
-        <v>1</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4">
-        <v>1</v>
-      </c>
-      <c r="K6" s="4">
-        <v>0</v>
-      </c>
-      <c r="L6" s="4">
-        <v>0</v>
-      </c>
-      <c r="M6" s="4">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4">
-        <v>0</v>
-      </c>
-      <c r="O6" s="4">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4">
-        <v>0</v>
-      </c>
-      <c r="S6" s="4">
-        <v>0</v>
-      </c>
-      <c r="T6" s="4">
-        <v>0</v>
-      </c>
-      <c r="U6" s="4">
-        <v>0</v>
-      </c>
-      <c r="V6" s="4">
+      <c r="B8" s="4">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4">
+        <v>0</v>
+      </c>
+      <c r="P8" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4">
+        <v>0</v>
+      </c>
+      <c r="T8" s="4">
+        <v>0</v>
+      </c>
+      <c r="U8" s="4">
+        <v>0</v>
+      </c>
+      <c r="V8" s="4">
+        <v>0</v>
+      </c>
+      <c r="W8" s="4">
+        <v>0</v>
+      </c>
+      <c r="X8" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
-        <v>0</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4">
-        <v>0</v>
-      </c>
-      <c r="I7" s="4">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4">
-        <v>0</v>
-      </c>
-      <c r="K7" s="4">
-        <v>1</v>
-      </c>
-      <c r="L7" s="4">
-        <v>1</v>
-      </c>
-      <c r="M7" s="4">
-        <v>1</v>
-      </c>
-      <c r="N7" s="4">
-        <v>0</v>
-      </c>
-      <c r="O7" s="4">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="4">
-        <v>0</v>
-      </c>
-      <c r="R7" s="4">
-        <v>0</v>
-      </c>
-      <c r="S7" s="4">
-        <v>0</v>
-      </c>
-      <c r="T7" s="4">
-        <v>0</v>
-      </c>
-      <c r="U7" s="4">
-        <v>0</v>
-      </c>
-      <c r="V7" s="4">
+      <c r="B9" s="4">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4">
+        <v>0</v>
+      </c>
+      <c r="N9" s="4">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4">
+        <v>1</v>
+      </c>
+      <c r="R9" s="4">
+        <v>1</v>
+      </c>
+      <c r="S9" s="4">
+        <v>1</v>
+      </c>
+      <c r="T9" s="4">
+        <v>0</v>
+      </c>
+      <c r="U9" s="4">
+        <v>0</v>
+      </c>
+      <c r="V9" s="4">
+        <v>0</v>
+      </c>
+      <c r="W9" s="4">
+        <v>0</v>
+      </c>
+      <c r="X9" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4">
-        <v>0</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4">
-        <v>0</v>
-      </c>
-      <c r="M8" s="4">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4">
-        <v>1</v>
-      </c>
-      <c r="O8" s="4">
-        <v>1</v>
-      </c>
-      <c r="P8" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="4">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4">
-        <v>0</v>
-      </c>
-      <c r="T8" s="4">
-        <v>0</v>
-      </c>
-      <c r="U8" s="4">
-        <v>0</v>
-      </c>
-      <c r="V8" s="4">
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4">
+        <v>0</v>
+      </c>
+      <c r="T10" s="4">
+        <v>1</v>
+      </c>
+      <c r="U10" s="4">
+        <v>1</v>
+      </c>
+      <c r="V10" s="4">
+        <v>0</v>
+      </c>
+      <c r="W10" s="4">
+        <v>0</v>
+      </c>
+      <c r="X10" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4">
-        <v>0</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4">
-        <v>0</v>
-      </c>
-      <c r="K9" s="4">
-        <v>0</v>
-      </c>
-      <c r="L9" s="4">
-        <v>0</v>
-      </c>
-      <c r="M9" s="4">
-        <v>0</v>
-      </c>
-      <c r="N9" s="4">
-        <v>0</v>
-      </c>
-      <c r="O9" s="4">
-        <v>0</v>
-      </c>
-      <c r="P9" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="4">
-        <v>0</v>
-      </c>
-      <c r="R9" s="4">
-        <v>0</v>
-      </c>
-      <c r="S9" s="4">
-        <v>0</v>
-      </c>
-      <c r="T9" s="4">
-        <v>0</v>
-      </c>
-      <c r="U9" s="4">
-        <v>0</v>
-      </c>
-      <c r="V9" s="4">
+      <c r="B11" s="4">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4">
+        <v>0</v>
+      </c>
+      <c r="T11" s="4">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4">
+        <v>0</v>
+      </c>
+      <c r="V11" s="4">
+        <v>1</v>
+      </c>
+      <c r="W11" s="4">
+        <v>0</v>
+      </c>
+      <c r="X11" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="4">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4">
-        <v>0</v>
-      </c>
-      <c r="J10" s="4">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4">
-        <v>0</v>
-      </c>
-      <c r="L10" s="4">
-        <v>0</v>
-      </c>
-      <c r="M10" s="4">
-        <v>0</v>
-      </c>
-      <c r="N10" s="4">
-        <v>0</v>
-      </c>
-      <c r="O10" s="4">
-        <v>0</v>
-      </c>
-      <c r="P10" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="4">
-        <v>1</v>
-      </c>
-      <c r="R10" s="4">
-        <v>0</v>
-      </c>
-      <c r="S10" s="4">
-        <v>0</v>
-      </c>
-      <c r="T10" s="4">
-        <v>0</v>
-      </c>
-      <c r="U10" s="4">
-        <v>0</v>
-      </c>
-      <c r="V10" s="4">
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4">
+        <v>0</v>
+      </c>
+      <c r="T12" s="4">
+        <v>0</v>
+      </c>
+      <c r="U12" s="4">
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
+        <v>0</v>
+      </c>
+      <c r="W12" s="4">
+        <v>1</v>
+      </c>
+      <c r="X12" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="4">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4">
-        <v>0</v>
-      </c>
-      <c r="E11" s="4">
-        <v>0</v>
-      </c>
-      <c r="F11" s="4">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4">
-        <v>0</v>
-      </c>
-      <c r="I11" s="4">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4">
-        <v>0</v>
-      </c>
-      <c r="L11" s="4">
-        <v>0</v>
-      </c>
-      <c r="M11" s="4">
-        <v>0</v>
-      </c>
-      <c r="N11" s="4">
-        <v>0</v>
-      </c>
-      <c r="O11" s="4">
-        <v>0</v>
-      </c>
-      <c r="P11" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="4">
-        <v>0</v>
-      </c>
-      <c r="R11" s="4">
-        <v>1</v>
-      </c>
-      <c r="S11" s="4">
-        <v>1</v>
-      </c>
-      <c r="T11" s="4">
-        <v>0</v>
-      </c>
-      <c r="U11" s="4">
-        <v>0</v>
-      </c>
-      <c r="V11" s="4">
+      <c r="B13" s="4">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4">
+        <v>0</v>
+      </c>
+      <c r="R13" s="4">
+        <v>0</v>
+      </c>
+      <c r="S13" s="4">
+        <v>0</v>
+      </c>
+      <c r="T13" s="4">
+        <v>0</v>
+      </c>
+      <c r="U13" s="4">
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
+        <v>0</v>
+      </c>
+      <c r="W13" s="4">
+        <v>0</v>
+      </c>
+      <c r="X13" s="4">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="4">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4">
-        <v>0</v>
-      </c>
-      <c r="L12" s="4">
-        <v>0</v>
-      </c>
-      <c r="M12" s="4">
-        <v>0</v>
-      </c>
-      <c r="N12" s="4">
-        <v>0</v>
-      </c>
-      <c r="O12" s="4">
-        <v>0</v>
-      </c>
-      <c r="P12" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="4">
-        <v>0</v>
-      </c>
-      <c r="R12" s="4">
-        <v>0</v>
-      </c>
-      <c r="S12" s="4">
-        <v>0</v>
-      </c>
-      <c r="T12" s="4">
-        <v>1</v>
-      </c>
-      <c r="U12" s="4">
-        <v>0</v>
-      </c>
-      <c r="V12" s="4">
+      <c r="B14" s="4">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
+        <v>0</v>
+      </c>
+      <c r="M14" s="4">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4">
+        <v>0</v>
+      </c>
+      <c r="R14" s="4">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4">
+        <v>0</v>
+      </c>
+      <c r="T14" s="4">
+        <v>0</v>
+      </c>
+      <c r="U14" s="4">
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
+        <v>0</v>
+      </c>
+      <c r="W14" s="4">
+        <v>0</v>
+      </c>
+      <c r="X14" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="4">
-        <v>0</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4">
-        <v>0</v>
-      </c>
-      <c r="E13" s="4">
-        <v>0</v>
-      </c>
-      <c r="F13" s="4">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4">
-        <v>0</v>
-      </c>
-      <c r="I13" s="4">
-        <v>0</v>
-      </c>
-      <c r="J13" s="4">
-        <v>0</v>
-      </c>
-      <c r="K13" s="4">
-        <v>0</v>
-      </c>
-      <c r="L13" s="4">
-        <v>0</v>
-      </c>
-      <c r="M13" s="4">
-        <v>0</v>
-      </c>
-      <c r="N13" s="4">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4">
-        <v>0</v>
-      </c>
-      <c r="P13" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="4">
-        <v>0</v>
-      </c>
-      <c r="R13" s="4">
-        <v>0</v>
-      </c>
-      <c r="S13" s="4">
-        <v>0</v>
-      </c>
-      <c r="T13" s="4">
-        <v>0</v>
-      </c>
-      <c r="U13" s="4">
-        <v>1</v>
-      </c>
-      <c r="V13" s="4">
+      <c r="B15" s="4">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4">
+        <v>0</v>
+      </c>
+      <c r="N15" s="4">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4">
+        <v>0</v>
+      </c>
+      <c r="P15" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="4">
+        <v>0</v>
+      </c>
+      <c r="R15" s="4">
+        <v>0</v>
+      </c>
+      <c r="S15" s="4">
+        <v>0</v>
+      </c>
+      <c r="T15" s="4">
+        <v>0</v>
+      </c>
+      <c r="U15" s="4">
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
+        <v>0</v>
+      </c>
+      <c r="W15" s="4">
+        <v>0</v>
+      </c>
+      <c r="X15" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB15" s="4">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:V13">
+  <conditionalFormatting sqref="B2:AB15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>

</xml_diff>